<commit_message>
Added the Methane CH4 , LDR, Temp/Hum and H2S Sensor
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP i7\OneDrive\Desktop\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Plant Monitoring Sensor Network\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9345" windowHeight="6330" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9345" windowHeight="6330"/>
   </bookViews>
   <sheets>
     <sheet name="Adafruit" sheetId="6" r:id="rId1"/>
@@ -671,12 +671,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -692,7 +698,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -703,6 +709,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1027,7 +1034,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C2" t="s">
@@ -1079,7 +1086,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C4" t="s">
@@ -1105,7 +1112,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C5" t="s">
@@ -1131,7 +1138,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">

</xml_diff>